<commit_message>
Finished powerbi viz, need to do README
</commit_message>
<xml_diff>
--- a/student performance analysis.xlsx
+++ b/student performance analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programe\Programare\Data Analysis\Student Performance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72B7B7E1-A88A-4CDA-9A2E-3DC8994DCF0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7866C488-7036-4A40-8D41-4C75BED3E83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="37" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -1199,6 +1199,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-8DAF-4EE5-BF14-C77F6ABEEA33}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="1"/>
@@ -1216,6 +1221,11 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-8DAF-4EE5-BF14-C77F6ABEEA33}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:spPr>
@@ -5786,8 +5796,8 @@
       <xdr:row>9</xdr:row>
       <xdr:rowOff>57150</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="3" name="Is the student prepared?">
@@ -5810,7 +5820,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -5864,8 +5874,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>28575</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="4" name="Gender Of Student">
@@ -5888,7 +5898,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -5942,8 +5952,8 @@
       <xdr:row>23</xdr:row>
       <xdr:rowOff>38100</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="5" name="Parent's nivel of education">
@@ -5966,7 +5976,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -6020,8 +6030,8 @@
       <xdr:row>34</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:graphicFrame macro="">
           <xdr:nvGraphicFramePr>
             <xdr:cNvPr id="6" name="has passed">
@@ -6044,7 +6054,7 @@
           </a:graphic>
         </xdr:graphicFrame>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="0" name=""/>
@@ -20775,7 +20785,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAD7621D-D3C0-4BCF-89B4-EC09D4AAB8F8}" name="Student Scores" cacheId="37" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Student ID">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{AAD7621D-D3C0-4BCF-89B4-EC09D4AAB8F8}" name="Student Scores" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" rowGrandTotals="0" colGrandTotals="0" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="10" rowHeaderCaption="Student ID">
   <location ref="A1:E1001" firstHeaderRow="0" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="11">
     <pivotField axis="axisRow" showAll="0">

</xml_diff>

<commit_message>
Fixed bugs, finished README.md
</commit_message>
<xml_diff>
--- a/student performance analysis.xlsx
+++ b/student performance analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programe\Programare\Data Analysis\Student Performance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7866C488-7036-4A40-8D41-4C75BED3E83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{425DA401-185A-4443-9409-088332E12208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -92,7 +92,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6060" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6064" uniqueCount="60">
   <si>
     <t>gender</t>
   </si>
@@ -255,12 +255,30 @@
   <si>
     <t>Female scores</t>
   </si>
+  <si>
+    <t>Passing Rate</t>
+  </si>
+  <si>
+    <t>Count of students that passed</t>
+  </si>
+  <si>
+    <t>Total count of students</t>
+  </si>
+  <si>
+    <t>Count of students that failed</t>
+  </si>
+  <si>
+    <t>The Smallest Reading Score</t>
+  </si>
+  <si>
+    <t>The Smallest Writing Score</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -275,8 +293,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -301,6 +326,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -311,10 +342,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -322,14 +354,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="2" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="2" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="10" fontId="0" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="8">
     <dxf>
@@ -2501,8 +2537,8 @@
   </c:txPr>
   <c:printSettings>
     <c:headerFooter/>
-    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
-    <c:pageSetup/>
+    <c:pageMargins b="0.74803149606299213" l="0.70866141732283472" r="0.70866141732283472" t="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
+    <c:pageSetup paperSize="9" orientation="landscape"/>
   </c:printSettings>
 </c:chartSpace>
 </file>
@@ -3182,6 +3218,289 @@
 </c:chartSpace>
 </file>
 
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="103"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="3"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Student's</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" baseline="0"/>
+              <a:t> rate of passing</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:shade val="76000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-1309-4FD4-8669-C6B7079D2D26}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1">
+                  <a:tint val="77000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:schemeClr val="lt1"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-1309-4FD4-8669-C6B7079D2D26}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:spPr>
+              <a:solidFill>
+                <a:sysClr val="window" lastClr="FFFFFF"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000">
+                    <a:lumMod val="25000"/>
+                    <a:lumOff val="75000"/>
+                  </a:sysClr>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="dk1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="1"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="1"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:spPr xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart">
+                  <a:prstGeom prst="wedgeRectCallout">
+                    <a:avLst/>
+                  </a:prstGeom>
+                  <a:noFill/>
+                  <a:ln>
+                    <a:noFill/>
+                  </a:ln>
+                </c15:spPr>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'Score Graphs'!$P$40:$Q$40</c:f>
+              <c:strCache>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>Count of students that passed</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Count of students that failed</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Score Graphs'!$P$41:$Q$41</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+                <c:pt idx="0">
+                  <c:v>812</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>188</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-054D-41AF-9E75-5BB2B5E2C1CD}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="0"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:solidFill>
+        <a:schemeClr val="tx1">
+          <a:lumMod val="15000"/>
+          <a:lumOff val="85000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
 <file path=xl/charts/colors1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
   <a:schemeClr val="accent1"/>
@@ -3241,6 +3560,12 @@
 </file>
 
 <file path=xl/charts/colors5.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
+  <a:schemeClr val="accent1"/>
+</cs:colorStyle>
+</file>
+
+<file path=xl/charts/colors6.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="14">
   <a:schemeClr val="accent1"/>
 </cs:colorStyle>
@@ -5781,6 +6106,525 @@
 </cs:chartStyle>
 </file>
 
+<file path=xl/charts/style6.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="251">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="25400">
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="75000"/>
+          <a:lumOff val="25000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="50000"/>
+            <a:lumOff val="50000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
@@ -6181,7 +7025,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>534361</xdr:colOff>
+      <xdr:colOff>210511</xdr:colOff>
       <xdr:row>15</xdr:row>
       <xdr:rowOff>85044</xdr:rowOff>
     </xdr:to>
@@ -6275,6 +7119,42 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>381000</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>36739</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>598714</xdr:colOff>
+      <xdr:row>38</xdr:row>
+      <xdr:rowOff>13607</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5390840E-3009-D72D-4BCD-57E684EF7C11}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -25263,6 +26143,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EE3BECB3-5D2A-4C06-AF75-4C0FD486D745}">
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
   <dimension ref="A1:L1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -61318,15 +62201,19 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FBB801F-37ED-4697-B0F7-44CD146392F9}">
-  <dimension ref="A1:L1001"/>
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:M1001"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
@@ -61342,7 +62229,7 @@
     <col min="1005" max="1005" width="11.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>28</v>
       </c>
@@ -61358,8 +62245,14 @@
       <c r="E1" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="M1" s="9"/>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>0</v>
       </c>
@@ -61375,12 +62268,18 @@
       <c r="E2" s="1">
         <v>74</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="L2" s="6"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L2" s="5"/>
+      <c r="M2" s="9"/>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>1</v>
       </c>
@@ -61396,14 +62295,20 @@
       <c r="E3" s="1">
         <v>88</v>
       </c>
-      <c r="K3" s="7" t="s">
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L3" s="7" t="s">
+      <c r="L3" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M3" s="9"/>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>2</v>
       </c>
@@ -61419,16 +62324,22 @@
       <c r="E4" s="1">
         <v>93</v>
       </c>
-      <c r="K4" s="8">
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="7">
         <f>_xlfn.XLOOKUP(L4,$B$2:$B$1001,$A$2:$A$1001)</f>
         <v>458</v>
       </c>
-      <c r="L4" s="9">
+      <c r="L4" s="8">
         <f>MAX(B:B)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M4" s="9"/>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>3</v>
       </c>
@@ -61444,12 +62355,16 @@
       <c r="E5" s="1">
         <v>44</v>
       </c>
-      <c r="I5" s="5"/>
-      <c r="J5" s="5"/>
-      <c r="K5" s="5"/>
-      <c r="L5" s="5"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="12"/>
+      <c r="J5" s="12"/>
+      <c r="K5" s="12"/>
+      <c r="L5" s="12"/>
+      <c r="M5" s="9"/>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>4</v>
       </c>
@@ -61465,13 +62380,18 @@
       <c r="E6" s="1">
         <v>75</v>
       </c>
-      <c r="J6" s="5"/>
-      <c r="K6" s="6" t="s">
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="12"/>
+      <c r="K6" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="L6" s="6"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L6" s="5"/>
+      <c r="M6" s="9"/>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>5</v>
       </c>
@@ -61487,15 +62407,20 @@
       <c r="E7" s="1">
         <v>78</v>
       </c>
-      <c r="J7" s="5"/>
-      <c r="K7" s="7" t="s">
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="12"/>
+      <c r="K7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L7" s="7" t="s">
+      <c r="L7" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M7" s="9"/>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>6</v>
       </c>
@@ -61511,18 +62436,22 @@
       <c r="E8" s="1">
         <v>92</v>
       </c>
-      <c r="I8" s="5"/>
-      <c r="J8" s="5"/>
-      <c r="K8" s="8">
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="12"/>
+      <c r="J8" s="12"/>
+      <c r="K8" s="7">
         <f>_xlfn.XLOOKUP(L8,$B$2:$B$1001,$A$2:$A$1001)</f>
         <v>59</v>
       </c>
-      <c r="L8" s="9">
+      <c r="L8" s="8">
         <f>MIN(B:B)</f>
         <v>9</v>
       </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M8" s="9"/>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>7</v>
       </c>
@@ -61538,10 +62467,16 @@
       <c r="E9" s="1">
         <v>39</v>
       </c>
-      <c r="I9" s="5"/>
-      <c r="J9" s="5"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="12"/>
+      <c r="J9" s="12"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>8</v>
       </c>
@@ -61557,10 +62492,16 @@
       <c r="E10" s="1">
         <v>67</v>
       </c>
-      <c r="I10" s="5"/>
-      <c r="J10" s="5"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="12"/>
+      <c r="J10" s="12"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+    </row>
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>9</v>
       </c>
@@ -61576,12 +62517,18 @@
       <c r="E11" s="1">
         <v>50</v>
       </c>
-      <c r="K11" s="6" t="s">
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="L11" s="6"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L11" s="5"/>
+      <c r="M11" s="9"/>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>10</v>
       </c>
@@ -61597,14 +62544,20 @@
       <c r="E12" s="1">
         <v>52</v>
       </c>
-      <c r="K12" s="7" t="s">
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L12" s="7" t="s">
+      <c r="L12" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M12" s="9"/>
+    </row>
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>11</v>
       </c>
@@ -61620,16 +62573,22 @@
       <c r="E13" s="1">
         <v>43</v>
       </c>
-      <c r="K13" s="8">
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="7">
         <f>_xlfn.XLOOKUP(L13,$C$2:$C$1001,$A$2:$A$1001)</f>
         <v>149</v>
       </c>
-      <c r="L13" s="9">
+      <c r="L13" s="8">
         <f>MAX(C:C)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M13" s="9"/>
+    </row>
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>12</v>
       </c>
@@ -61645,10 +62604,16 @@
       <c r="E14" s="1">
         <v>73</v>
       </c>
-      <c r="K14" s="5"/>
-      <c r="L14" s="5"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="12"/>
+      <c r="L14" s="12"/>
+      <c r="M14" s="9"/>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>13</v>
       </c>
@@ -61664,12 +62629,18 @@
       <c r="E15" s="1">
         <v>70</v>
       </c>
-      <c r="K15" s="6" t="s">
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="L15" s="6"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L15" s="5"/>
+      <c r="M15" s="9"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>14</v>
       </c>
@@ -61685,14 +62656,20 @@
       <c r="E16" s="1">
         <v>58</v>
       </c>
-      <c r="K16" s="7" t="s">
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L16" s="7" t="s">
+      <c r="L16" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M16" s="9"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>15</v>
       </c>
@@ -61708,16 +62685,22 @@
       <c r="E17" s="1">
         <v>78</v>
       </c>
-      <c r="K17" s="8">
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="7">
         <f>_xlfn.XLOOKUP(L17,$C$2:$C$1001,$A$2:$A$1001)</f>
         <v>59</v>
       </c>
-      <c r="L17" s="9">
+      <c r="L17" s="8">
         <f>MIN(C:C)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M17" s="9"/>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>16</v>
       </c>
@@ -61733,8 +62716,16 @@
       <c r="E18" s="1">
         <v>86</v>
       </c>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9"/>
+      <c r="K18" s="9"/>
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>17</v>
       </c>
@@ -61750,8 +62741,16 @@
       <c r="E19" s="1">
         <v>28</v>
       </c>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9"/>
+      <c r="K19" s="9"/>
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>18</v>
       </c>
@@ -61767,12 +62766,18 @@
       <c r="E20" s="1">
         <v>46</v>
       </c>
-      <c r="K20" s="6" t="s">
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="L20" s="6"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L20" s="5"/>
+      <c r="M20" s="9"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>19</v>
       </c>
@@ -61788,14 +62793,20 @@
       <c r="E21" s="1">
         <v>61</v>
       </c>
-      <c r="K21" s="7" t="s">
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L21" s="7" t="s">
+      <c r="L21" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M21" s="9"/>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>20</v>
       </c>
@@ -61811,16 +62822,22 @@
       <c r="E22" s="1">
         <v>63</v>
       </c>
-      <c r="K22" s="8">
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="7">
         <f>_xlfn.XLOOKUP(L22,$D$2:$D$1001,$A$2:$A$1001)</f>
         <v>106</v>
       </c>
-      <c r="L22" s="9">
+      <c r="L22" s="8">
         <f>MAX(D:D)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M22" s="9"/>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>21</v>
       </c>
@@ -61836,10 +62853,16 @@
       <c r="E23" s="1">
         <v>70</v>
       </c>
-      <c r="K23" s="5"/>
-      <c r="L23" s="5"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="12"/>
+      <c r="L23" s="12"/>
+      <c r="M23" s="9"/>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>22</v>
       </c>
@@ -61855,12 +62878,18 @@
       <c r="E24" s="1">
         <v>53</v>
       </c>
-      <c r="K24" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L24" s="6"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="L24" s="5"/>
+      <c r="M24" s="9"/>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>23</v>
       </c>
@@ -61876,14 +62905,20 @@
       <c r="E25" s="1">
         <v>73</v>
       </c>
-      <c r="K25" s="7" t="s">
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L25" s="7" t="s">
+      <c r="L25" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M25" s="9"/>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>24</v>
       </c>
@@ -61899,16 +62934,22 @@
       <c r="E26" s="1">
         <v>80</v>
       </c>
-      <c r="K26" s="8">
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="7">
         <f>_xlfn.XLOOKUP(L26,$D$2:$D$1001,$A$2:$A$1001)</f>
         <v>59</v>
       </c>
-      <c r="L26" s="9">
+      <c r="L26" s="8">
         <f>MIN(D:D)</f>
         <v>17</v>
       </c>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M26" s="9"/>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>25</v>
       </c>
@@ -61924,8 +62965,16 @@
       <c r="E27" s="1">
         <v>72</v>
       </c>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>26</v>
       </c>
@@ -61941,8 +62990,16 @@
       <c r="E28" s="1">
         <v>55</v>
       </c>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>27</v>
       </c>
@@ -61958,12 +63015,18 @@
       <c r="E29" s="1">
         <v>75</v>
       </c>
-      <c r="K29" s="6" t="s">
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="L29" s="6"/>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L29" s="5"/>
+      <c r="M29" s="9"/>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>28</v>
       </c>
@@ -61979,14 +63042,20 @@
       <c r="E30" s="1">
         <v>65</v>
       </c>
-      <c r="K30" s="7" t="s">
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L30" s="7" t="s">
+      <c r="L30" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M30" s="9"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>29</v>
       </c>
@@ -62002,16 +63071,22 @@
       <c r="E31" s="1">
         <v>75</v>
       </c>
-      <c r="K31" s="8">
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="7">
         <f>_xlfn.XLOOKUP(L31,$E$2:$E$1001,$A$2:$A$1001)</f>
         <v>106</v>
       </c>
-      <c r="L31" s="9">
+      <c r="L31" s="8">
         <f>MAX(E:E)</f>
         <v>100</v>
       </c>
-    </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M31" s="9"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>30</v>
       </c>
@@ -62027,10 +63102,16 @@
       <c r="E32" s="1">
         <v>74</v>
       </c>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="12"/>
+      <c r="L32" s="12"/>
+      <c r="M32" s="9"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>31</v>
       </c>
@@ -62046,12 +63127,18 @@
       <c r="E33" s="1">
         <v>61</v>
       </c>
-      <c r="K33" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="L33" s="6"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="L33" s="5"/>
+      <c r="M33" s="9"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>32</v>
       </c>
@@ -62067,14 +63154,20 @@
       <c r="E34" s="1">
         <v>65</v>
       </c>
-      <c r="K34" s="7" t="s">
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="L34" s="7" t="s">
+      <c r="L34" s="6" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M34" s="9"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>33</v>
       </c>
@@ -62090,16 +63183,22 @@
       <c r="E35" s="1">
         <v>38</v>
       </c>
-      <c r="K35" s="8">
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="7">
         <f>_xlfn.XLOOKUP(L35,$E$2:$E$1001,$A$2:$A$1001)</f>
         <v>59</v>
       </c>
-      <c r="L35" s="9">
+      <c r="L35" s="8">
         <f>MIN(E:E)</f>
         <v>10</v>
       </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M35" s="9"/>
+    </row>
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>34</v>
       </c>
@@ -62115,8 +63214,16 @@
       <c r="E36" s="1">
         <v>82</v>
       </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>35</v>
       </c>
@@ -62132,8 +63239,16 @@
       <c r="E37" s="1">
         <v>79</v>
       </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="9"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
+      <c r="L37" s="9"/>
+      <c r="M37" s="9"/>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
         <v>36</v>
       </c>
@@ -62149,8 +63264,16 @@
       <c r="E38" s="1">
         <v>83</v>
       </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
         <v>37</v>
       </c>
@@ -62166,8 +63289,16 @@
       <c r="E39" s="1">
         <v>59</v>
       </c>
-    </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
+      <c r="K39" s="9"/>
+      <c r="L39" s="9"/>
+      <c r="M39" s="9"/>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>38</v>
       </c>
@@ -62183,8 +63314,16 @@
       <c r="E40" s="1">
         <v>88</v>
       </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" s="9"/>
+      <c r="K40" s="9"/>
+      <c r="L40" s="9"/>
+      <c r="M40" s="9"/>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>39</v>
       </c>
@@ -62200,8 +63339,16 @@
       <c r="E41" s="1">
         <v>57</v>
       </c>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+      <c r="I41" s="9"/>
+      <c r="J41" s="9"/>
+      <c r="K41" s="9"/>
+      <c r="L41" s="9"/>
+      <c r="M41" s="9"/>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>40</v>
       </c>
@@ -62217,8 +63364,12 @@
       <c r="E42" s="1">
         <v>54</v>
       </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+      <c r="J42" s="9"/>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>41</v>
       </c>
@@ -62235,7 +63386,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
         <v>42</v>
       </c>
@@ -62252,7 +63403,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>43</v>
       </c>
@@ -62269,7 +63420,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>44</v>
       </c>
@@ -62286,7 +63437,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>45</v>
       </c>
@@ -62303,7 +63454,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>46</v>
       </c>
@@ -78523,11 +79674,12 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
+  <drawing r:id="rId3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">
       <x14:slicerList>
-        <x14:slicer r:id="rId3"/>
+        <x14:slicer r:id="rId4"/>
       </x14:slicerList>
     </ext>
   </extLst>
@@ -78536,7 +79688,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95ED0464-0B32-44C5-A3B2-C1CF4F8B7C0C}">
-  <dimension ref="B18:Q44"/>
+  <sheetPr>
+    <pageSetUpPr autoPageBreaks="0"/>
+  </sheetPr>
+  <dimension ref="A1:T46"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
@@ -78548,288 +79703,1231 @@
     <col min="11" max="11" width="22" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="25.85546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="27.85546875" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="31.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="C18" t="s">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A1" s="9"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+      <c r="I1" s="9"/>
+      <c r="J1" s="9"/>
+      <c r="K1" s="9"/>
+      <c r="L1" s="9"/>
+      <c r="M1" s="9"/>
+      <c r="N1" s="9"/>
+      <c r="O1" s="9"/>
+      <c r="P1" s="9"/>
+      <c r="Q1" s="9"/>
+      <c r="R1" s="9"/>
+      <c r="S1" s="9"/>
+      <c r="T1" s="9"/>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A2" s="9"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="9"/>
+      <c r="J2" s="9"/>
+      <c r="K2" s="9"/>
+      <c r="L2" s="9"/>
+      <c r="M2" s="9"/>
+      <c r="N2" s="9"/>
+      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
+      <c r="Q2" s="9"/>
+      <c r="R2" s="9"/>
+      <c r="S2" s="9"/>
+      <c r="T2" s="9"/>
+    </row>
+    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
+      <c r="I3" s="9"/>
+      <c r="J3" s="9"/>
+      <c r="K3" s="9"/>
+      <c r="L3" s="9"/>
+      <c r="M3" s="9"/>
+      <c r="N3" s="9"/>
+      <c r="O3" s="9"/>
+      <c r="P3" s="9"/>
+      <c r="Q3" s="9"/>
+      <c r="R3" s="9"/>
+      <c r="S3" s="9"/>
+      <c r="T3" s="9"/>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
+      <c r="I4" s="9"/>
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+    </row>
+    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
+      <c r="I5" s="9"/>
+      <c r="J5" s="9"/>
+      <c r="K5" s="9"/>
+      <c r="L5" s="9"/>
+      <c r="M5" s="9"/>
+      <c r="N5" s="9"/>
+      <c r="O5" s="9"/>
+      <c r="P5" s="9"/>
+      <c r="Q5" s="9"/>
+      <c r="R5" s="9"/>
+      <c r="S5" s="9"/>
+      <c r="T5" s="9"/>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A6" s="9"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+      <c r="H6" s="9"/>
+      <c r="I6" s="9"/>
+      <c r="J6" s="9"/>
+      <c r="K6" s="9"/>
+      <c r="L6" s="9"/>
+      <c r="M6" s="9"/>
+      <c r="N6" s="9"/>
+      <c r="O6" s="9"/>
+      <c r="P6" s="9"/>
+      <c r="Q6" s="9"/>
+      <c r="R6" s="9"/>
+      <c r="S6" s="9"/>
+      <c r="T6" s="9"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A7" s="9"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9"/>
+      <c r="M7" s="9"/>
+      <c r="N7" s="9"/>
+      <c r="O7" s="9"/>
+      <c r="P7" s="9"/>
+      <c r="Q7" s="9"/>
+      <c r="R7" s="9"/>
+      <c r="S7" s="9"/>
+      <c r="T7" s="9"/>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A8" s="9"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+      <c r="L8" s="9"/>
+      <c r="M8" s="9"/>
+      <c r="N8" s="9"/>
+      <c r="O8" s="9"/>
+      <c r="P8" s="9"/>
+      <c r="Q8" s="9"/>
+      <c r="R8" s="9"/>
+      <c r="S8" s="9"/>
+      <c r="T8" s="9"/>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A9" s="9"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+      <c r="L9" s="9"/>
+      <c r="M9" s="9"/>
+      <c r="N9" s="9"/>
+      <c r="O9" s="9"/>
+      <c r="P9" s="9"/>
+      <c r="Q9" s="9"/>
+      <c r="R9" s="9"/>
+      <c r="S9" s="9"/>
+      <c r="T9" s="9"/>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A10" s="9"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+      <c r="L10" s="9"/>
+      <c r="M10" s="9"/>
+      <c r="N10" s="9"/>
+      <c r="O10" s="9"/>
+      <c r="P10" s="9"/>
+      <c r="Q10" s="9"/>
+      <c r="R10" s="9"/>
+      <c r="S10" s="9"/>
+      <c r="T10" s="9"/>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A11" s="9"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+      <c r="L11" s="9"/>
+      <c r="M11" s="9"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="9"/>
+      <c r="P11" s="9"/>
+      <c r="Q11" s="9"/>
+      <c r="R11" s="9"/>
+      <c r="S11" s="9"/>
+      <c r="T11" s="9"/>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A12" s="9"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+      <c r="L12" s="9"/>
+      <c r="M12" s="9"/>
+      <c r="N12" s="9"/>
+      <c r="O12" s="9"/>
+      <c r="P12" s="9"/>
+      <c r="Q12" s="9"/>
+      <c r="R12" s="9"/>
+      <c r="S12" s="9"/>
+      <c r="T12" s="9"/>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A13" s="9"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+      <c r="L13" s="9"/>
+      <c r="M13" s="9"/>
+      <c r="N13" s="9"/>
+      <c r="O13" s="9"/>
+      <c r="P13" s="9"/>
+      <c r="Q13" s="9"/>
+      <c r="R13" s="9"/>
+      <c r="S13" s="9"/>
+      <c r="T13" s="9"/>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+      <c r="L14" s="9"/>
+      <c r="M14" s="9"/>
+      <c r="N14" s="9"/>
+      <c r="O14" s="9"/>
+      <c r="P14" s="9"/>
+      <c r="Q14" s="9"/>
+      <c r="R14" s="9"/>
+      <c r="S14" s="9"/>
+      <c r="T14" s="9"/>
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
+      <c r="L15" s="9"/>
+      <c r="M15" s="9"/>
+      <c r="N15" s="9"/>
+      <c r="O15" s="9"/>
+      <c r="P15" s="9"/>
+      <c r="Q15" s="9"/>
+      <c r="R15" s="9"/>
+      <c r="S15" s="9"/>
+      <c r="T15" s="9"/>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+      <c r="I16" s="9"/>
+      <c r="J16" s="9"/>
+      <c r="K16" s="9"/>
+      <c r="L16" s="9"/>
+      <c r="M16" s="9"/>
+      <c r="N16" s="9"/>
+      <c r="O16" s="9"/>
+      <c r="P16" s="9"/>
+      <c r="Q16" s="9"/>
+      <c r="R16" s="9"/>
+      <c r="S16" s="9"/>
+      <c r="T16" s="9"/>
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A17" s="9"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+      <c r="I17" s="9"/>
+      <c r="J17" s="9"/>
+      <c r="K17" s="9"/>
+      <c r="L17" s="9"/>
+      <c r="M17" s="9"/>
+      <c r="N17" s="9"/>
+      <c r="O17" s="9"/>
+      <c r="P17" s="9"/>
+      <c r="Q17" s="9"/>
+      <c r="R17" s="9"/>
+      <c r="S17" s="9"/>
+      <c r="T17" s="9"/>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A18" s="9"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="J18" t="s">
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+      <c r="I18" s="9"/>
+      <c r="J18" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="P18" t="s">
+      <c r="L18" s="9"/>
+      <c r="M18" s="9"/>
+      <c r="N18" s="9"/>
+      <c r="O18" s="9"/>
+      <c r="P18" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="Q18" s="9" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B19" t="s">
+      <c r="R18" s="9"/>
+      <c r="S18" s="9"/>
+      <c r="T18" s="9"/>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A19" s="9"/>
+      <c r="B19" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C19" s="2" cm="1">
+      <c r="C19" s="10" cm="1">
         <f t="array" ref="C19">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score],StudentsPerformance[has passed]="PASSED"))</f>
         <v>72.561986863710999</v>
       </c>
-      <c r="D19" s="2" cm="1">
+      <c r="D19" s="10" cm="1">
         <f t="array" ref="D19">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score],StudentsPerformance[has passed]="FAILED"))</f>
         <v>47.076241134751783</v>
       </c>
-      <c r="J19">
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+      <c r="I19" s="9"/>
+      <c r="J19" s="9">
         <f>COUNTIF(StudentsPerformance!B:B,"male")</f>
         <v>482</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="9">
         <f>COUNTIF(StudentsPerformance!$B:$B,"female")</f>
         <v>518</v>
       </c>
-      <c r="P19">
+      <c r="L19" s="9"/>
+      <c r="M19" s="9"/>
+      <c r="N19" s="9"/>
+      <c r="O19" s="9"/>
+      <c r="P19" s="9">
         <f>COUNTIF(StudentsPerformance!$F:$F, "completed")</f>
         <v>358</v>
       </c>
-      <c r="Q19">
+      <c r="Q19" s="9">
         <f>COUNTIF(StudentsPerformance!$F:$F, "none")</f>
         <v>642</v>
       </c>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B20" t="s">
+      <c r="R19" s="9"/>
+      <c r="S19" s="9"/>
+      <c r="T19" s="9"/>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A20" s="9"/>
+      <c r="B20" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="2" cm="1">
+      <c r="C20" s="10" cm="1">
         <f t="array" ref="C20">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score],StudentsPerformance[has passed]="PASSED"))</f>
         <v>70.949507389162562</v>
       </c>
-      <c r="D20" s="2" cm="1">
+      <c r="D20" s="10" cm="1">
         <f t="array" ref="D20">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score],StudentsPerformance[has passed]="FAILED"))</f>
         <v>45.095744680851062</v>
       </c>
-    </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+      <c r="I20" s="9"/>
+      <c r="J20" s="9"/>
+      <c r="K20" s="9"/>
+      <c r="L20" s="9"/>
+      <c r="M20" s="9"/>
+      <c r="N20" s="9"/>
+      <c r="O20" s="9"/>
+      <c r="P20" s="9"/>
+      <c r="Q20" s="9"/>
+      <c r="R20" s="9"/>
+      <c r="S20" s="9"/>
+      <c r="T20" s="9"/>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A21" s="9"/>
+      <c r="B21" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C21" s="2" cm="1">
+      <c r="C21" s="10" cm="1">
         <f t="array" ref="C21">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score],StudentsPerformance[has passed]="PASSED"))</f>
         <v>72.950738916256157</v>
       </c>
-      <c r="D21" s="2" cm="1">
+      <c r="D21" s="10" cm="1">
         <f t="array" ref="D21">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score],StudentsPerformance[has passed]="FAILED"))</f>
         <v>46.904255319148938</v>
       </c>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="B22" t="s">
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="9"/>
+      <c r="L21" s="9"/>
+      <c r="M21" s="9"/>
+      <c r="N21" s="9"/>
+      <c r="O21" s="9"/>
+      <c r="P21" s="9"/>
+      <c r="Q21" s="9"/>
+      <c r="R21" s="9"/>
+      <c r="S21" s="9"/>
+      <c r="T21" s="9"/>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A22" s="9"/>
+      <c r="B22" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C22" s="2" cm="1">
+      <c r="C22" s="10" cm="1">
         <f t="array" ref="C22">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score],StudentsPerformance[has passed]="PASSED"))</f>
         <v>73.785714285714292</v>
       </c>
-      <c r="D22" s="2" cm="1">
+      <c r="D22" s="10" cm="1">
         <f t="array" ref="D22">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score],StudentsPerformance[has passed]="FAILED"))</f>
         <v>49.228723404255319</v>
       </c>
-    </row>
-    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="C40" t="s">
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+      <c r="I22" s="9"/>
+      <c r="J22" s="9"/>
+      <c r="K22" s="9"/>
+      <c r="L22" s="9"/>
+      <c r="M22" s="9"/>
+      <c r="N22" s="9"/>
+      <c r="O22" s="9"/>
+      <c r="P22" s="9"/>
+      <c r="Q22" s="9"/>
+      <c r="R22" s="9"/>
+      <c r="S22" s="9"/>
+      <c r="T22" s="9"/>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+      <c r="I23" s="9"/>
+      <c r="J23" s="9"/>
+      <c r="K23" s="9"/>
+      <c r="L23" s="9"/>
+      <c r="M23" s="9"/>
+      <c r="N23" s="9"/>
+      <c r="O23" s="9"/>
+      <c r="P23" s="9"/>
+      <c r="Q23" s="9"/>
+      <c r="R23" s="9"/>
+      <c r="S23" s="9"/>
+      <c r="T23" s="9"/>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="9"/>
+      <c r="L24" s="9"/>
+      <c r="M24" s="9"/>
+      <c r="N24" s="9"/>
+      <c r="O24" s="9"/>
+      <c r="P24" s="9"/>
+      <c r="Q24" s="9"/>
+      <c r="R24" s="9"/>
+      <c r="S24" s="9"/>
+      <c r="T24" s="9"/>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+      <c r="I25" s="9"/>
+      <c r="J25" s="9"/>
+      <c r="K25" s="9"/>
+      <c r="L25" s="9"/>
+      <c r="M25" s="9"/>
+      <c r="N25" s="9"/>
+      <c r="O25" s="9"/>
+      <c r="P25" s="9"/>
+      <c r="Q25" s="9"/>
+      <c r="R25" s="9"/>
+      <c r="S25" s="9"/>
+      <c r="T25" s="9"/>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+      <c r="I26" s="9"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+      <c r="O26" s="9"/>
+      <c r="P26" s="9"/>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9"/>
+      <c r="S26" s="9"/>
+      <c r="T26" s="9"/>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+      <c r="I27" s="9"/>
+      <c r="J27" s="9"/>
+      <c r="K27" s="9"/>
+      <c r="L27" s="9"/>
+      <c r="M27" s="9"/>
+      <c r="N27" s="9"/>
+      <c r="O27" s="9"/>
+      <c r="P27" s="9"/>
+      <c r="Q27" s="9"/>
+      <c r="R27" s="9"/>
+      <c r="S27" s="9"/>
+      <c r="T27" s="9"/>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="9"/>
+      <c r="L28" s="9"/>
+      <c r="M28" s="9"/>
+      <c r="N28" s="9"/>
+      <c r="O28" s="9"/>
+      <c r="P28" s="9"/>
+      <c r="Q28" s="9"/>
+      <c r="R28" s="9"/>
+      <c r="S28" s="9"/>
+      <c r="T28" s="9"/>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+      <c r="I29" s="9"/>
+      <c r="J29" s="9"/>
+      <c r="K29" s="9"/>
+      <c r="L29" s="9"/>
+      <c r="M29" s="9"/>
+      <c r="N29" s="9"/>
+      <c r="O29" s="9"/>
+      <c r="P29" s="9"/>
+      <c r="Q29" s="9"/>
+      <c r="R29" s="9"/>
+      <c r="S29" s="9"/>
+      <c r="T29" s="9"/>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+      <c r="I30" s="9"/>
+      <c r="J30" s="9"/>
+      <c r="K30" s="9"/>
+      <c r="L30" s="9"/>
+      <c r="M30" s="9"/>
+      <c r="N30" s="9"/>
+      <c r="O30" s="9"/>
+      <c r="P30" s="9"/>
+      <c r="Q30" s="9"/>
+      <c r="R30" s="9"/>
+      <c r="S30" s="9"/>
+      <c r="T30" s="9"/>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A31" s="9"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="9"/>
+      <c r="L31" s="9"/>
+      <c r="M31" s="9"/>
+      <c r="N31" s="9"/>
+      <c r="O31" s="9"/>
+      <c r="P31" s="9"/>
+      <c r="Q31" s="9"/>
+      <c r="R31" s="9"/>
+      <c r="S31" s="9"/>
+      <c r="T31" s="9"/>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A32" s="9"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+      <c r="I32" s="9"/>
+      <c r="J32" s="9"/>
+      <c r="K32" s="9"/>
+      <c r="L32" s="9"/>
+      <c r="M32" s="9"/>
+      <c r="N32" s="9"/>
+      <c r="O32" s="9"/>
+      <c r="P32" s="9"/>
+      <c r="Q32" s="9"/>
+      <c r="R32" s="9"/>
+      <c r="S32" s="9"/>
+      <c r="T32" s="9"/>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+      <c r="I33" s="9"/>
+      <c r="J33" s="9"/>
+      <c r="K33" s="9"/>
+      <c r="L33" s="9"/>
+      <c r="M33" s="9"/>
+      <c r="N33" s="9"/>
+      <c r="O33" s="9"/>
+      <c r="P33" s="9"/>
+      <c r="Q33" s="9"/>
+      <c r="R33" s="9"/>
+      <c r="S33" s="9"/>
+      <c r="T33" s="9"/>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A34" s="9"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="9"/>
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+      <c r="I34" s="9"/>
+      <c r="J34" s="9"/>
+      <c r="K34" s="9"/>
+      <c r="L34" s="9"/>
+      <c r="M34" s="9"/>
+      <c r="N34" s="9"/>
+      <c r="O34" s="9"/>
+      <c r="P34" s="9"/>
+      <c r="Q34" s="9"/>
+      <c r="R34" s="9"/>
+      <c r="S34" s="9"/>
+      <c r="T34" s="9"/>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A35" s="9"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A36" s="9"/>
+      <c r="B36" s="9"/>
+      <c r="C36" s="9"/>
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+      <c r="I36" s="9"/>
+      <c r="J36" s="9"/>
+      <c r="K36" s="9"/>
+      <c r="L36" s="9"/>
+      <c r="M36" s="9"/>
+      <c r="N36" s="9"/>
+      <c r="O36" s="9"/>
+      <c r="P36" s="9"/>
+      <c r="Q36" s="9"/>
+      <c r="R36" s="9"/>
+      <c r="S36" s="9"/>
+      <c r="T36" s="9"/>
+    </row>
+    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A37" s="9"/>
+      <c r="B37" s="9"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+      <c r="I37" s="9"/>
+      <c r="J37" s="9"/>
+      <c r="K37" s="9"/>
+      <c r="L37" s="9"/>
+      <c r="M37" s="9"/>
+      <c r="N37" s="9"/>
+      <c r="O37" s="9"/>
+      <c r="P37" s="9"/>
+      <c r="Q37" s="9"/>
+      <c r="R37" s="9"/>
+      <c r="S37" s="9"/>
+      <c r="T37" s="9"/>
+    </row>
+    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A38" s="9"/>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+      <c r="I38" s="9"/>
+      <c r="J38" s="9"/>
+      <c r="K38" s="9"/>
+      <c r="L38" s="9"/>
+      <c r="M38" s="9"/>
+      <c r="N38" s="9"/>
+      <c r="O38" s="9"/>
+      <c r="P38" s="9"/>
+      <c r="Q38" s="9"/>
+      <c r="R38" s="9"/>
+      <c r="S38" s="9"/>
+      <c r="T38" s="9"/>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A39" s="9"/>
+      <c r="B39" s="9"/>
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
+      <c r="K39" s="9"/>
+      <c r="L39" s="9"/>
+      <c r="M39" s="9"/>
+      <c r="N39" s="9"/>
+      <c r="O39" s="9"/>
+      <c r="P39" s="9"/>
+      <c r="Q39" s="9"/>
+      <c r="R39" s="9"/>
+      <c r="S39" s="9"/>
+      <c r="T39" s="9"/>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A40" s="9"/>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D40" t="s">
+      <c r="D40" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="H40" t="str" cm="1">
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9" t="str" cm="1">
         <f t="array" ref="H40:M40">TRANSPOSE(_xlfn.UNIQUE(StudentsPerformance[parental level of education]))</f>
         <v>bachelor's degree</v>
       </c>
-      <c r="I40" t="str">
+      <c r="I40" s="9" t="str">
         <v>some college</v>
       </c>
-      <c r="J40" t="str">
+      <c r="J40" s="9" t="str">
         <v>master's degree</v>
       </c>
-      <c r="K40" t="str">
+      <c r="K40" s="9" t="str">
         <v>associate's degree</v>
       </c>
-      <c r="L40" t="str">
+      <c r="L40" s="9" t="str">
         <v>high school</v>
       </c>
-      <c r="M40" t="str">
+      <c r="M40" s="9" t="str">
         <v>some high school</v>
       </c>
-    </row>
-    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B41" t="s">
+      <c r="N40" s="9"/>
+      <c r="O40" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="P40" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q40" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="R40" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="S40" s="9"/>
+      <c r="T40" s="9"/>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A41" s="9"/>
+      <c r="B41" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C41" s="2" cm="1">
+      <c r="C41" s="10" cm="1">
         <f t="array" ref="C41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score],StudentsPerformance[gender]="male"))</f>
         <v>65.837482710926707</v>
       </c>
-      <c r="D41" s="2" cm="1">
+      <c r="D41" s="10" cm="1">
         <f t="array" ref="D41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score],StudentsPerformance[gender]="female"))</f>
         <v>69.56949806949811</v>
       </c>
-      <c r="G41" t="s">
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="H41" cm="1">
+      <c r="H41" s="9" cm="1">
         <f t="array" ref="H41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score], StudentsPerformance[parental level of education]='Score Graphs'!$H$40))</f>
         <v>71.923728813559308</v>
       </c>
-      <c r="I41" cm="1">
+      <c r="I41" s="9" cm="1">
         <f t="array" ref="I41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score], StudentsPerformance[parental level of education]='Score Graphs'!$I$40))</f>
         <v>68.476401179940993</v>
       </c>
-      <c r="J41" cm="1">
+      <c r="J41" s="9" cm="1">
         <f t="array" ref="J41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score], StudentsPerformance[parental level of education]='Score Graphs'!$J$40))</f>
         <v>73.598870056497177</v>
       </c>
-      <c r="K41" cm="1">
+      <c r="K41" s="9" cm="1">
         <f t="array" ref="K41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score], StudentsPerformance[parental level of education]='Score Graphs'!K40))</f>
         <v>69.569069069069073</v>
       </c>
-      <c r="L41" cm="1">
+      <c r="L41" s="9" cm="1">
         <f t="array" ref="L41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score], StudentsPerformance[parental level of education]='Score Graphs'!L40))</f>
         <v>63.09693877551021</v>
       </c>
-      <c r="M41" cm="1">
+      <c r="M41" s="9" cm="1">
         <f t="array" ref="M41">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[average score], StudentsPerformance[parental level of education]='Score Graphs'!M40))</f>
         <v>65.108007448789607</v>
       </c>
-    </row>
-    <row r="42" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B42" t="s">
+      <c r="N41" s="9"/>
+      <c r="O41" s="11">
+        <f xml:space="preserve"> P41 / R41</f>
+        <v>0.81200000000000006</v>
+      </c>
+      <c r="P41" s="9">
+        <f xml:space="preserve"> COUNTIF(StudentsPerformance[has passed], "PASSED")</f>
+        <v>812</v>
+      </c>
+      <c r="Q41" s="9">
+        <f xml:space="preserve"> R41 - P41</f>
+        <v>188</v>
+      </c>
+      <c r="R41" s="9">
+        <f xml:space="preserve"> COUNTA(StudentsPerformance[has passed])</f>
+        <v>1000</v>
+      </c>
+      <c r="S41" s="9"/>
+      <c r="T41" s="9"/>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A42" s="9"/>
+      <c r="B42" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C42" s="2" cm="1">
+      <c r="C42" s="10" cm="1">
         <f t="array" ref="C42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score],StudentsPerformance[gender]="male"))</f>
         <v>68.72821576763485</v>
       </c>
-      <c r="D42" s="2" cm="1">
+      <c r="D42" s="10" cm="1">
         <f t="array" ref="D42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score],StudentsPerformance[gender]="female"))</f>
         <v>63.633204633204635</v>
       </c>
-      <c r="G42" t="s">
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="H42" cm="1">
+      <c r="H42" s="9" cm="1">
         <f t="array" ref="H42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score], StudentsPerformance[parental level of education]='Score Graphs'!$H$40))</f>
         <v>69.389830508474574</v>
       </c>
-      <c r="I42" cm="1">
+      <c r="I42" s="9" cm="1">
         <f t="array" ref="I42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score], StudentsPerformance[parental level of education]='Score Graphs'!$I$40))</f>
         <v>67.128318584070797</v>
       </c>
-      <c r="J42" cm="1">
+      <c r="J42" s="9" cm="1">
         <f t="array" ref="J42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score], StudentsPerformance[parental level of education]='Score Graphs'!$J$40))</f>
         <v>69.745762711864401</v>
       </c>
-      <c r="K42" cm="1">
+      <c r="K42" s="9" cm="1">
         <f t="array" ref="K42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score], StudentsPerformance[parental level of education]='Score Graphs'!$K$40))</f>
         <v>67.882882882882882</v>
       </c>
-      <c r="L42" cm="1">
+      <c r="L42" s="9" cm="1">
         <f t="array" ref="L42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score], StudentsPerformance[parental level of education]='Score Graphs'!$L$40))</f>
         <v>62.137755102040813</v>
       </c>
-      <c r="M42" cm="1">
+      <c r="M42" s="9" cm="1">
         <f t="array" ref="M42">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[math score], StudentsPerformance[parental level of education]='Score Graphs'!$M$40))</f>
         <v>63.497206703910614</v>
       </c>
-    </row>
-    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B43" t="s">
+      <c r="N42" s="9"/>
+      <c r="O42" s="9"/>
+      <c r="P42" s="9"/>
+      <c r="Q42" s="9"/>
+      <c r="R42" s="9"/>
+      <c r="S42" s="9"/>
+      <c r="T42" s="9"/>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A43" s="9"/>
+      <c r="B43" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C43" s="2" cm="1">
+      <c r="C43" s="10" cm="1">
         <f t="array" ref="C43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score],StudentsPerformance[gender]="male"))</f>
         <v>63.311203319502077</v>
       </c>
-      <c r="D43" s="2" cm="1">
+      <c r="D43" s="10" cm="1">
         <f t="array" ref="D43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score],StudentsPerformance[gender]="female"))</f>
         <v>72.467181467181462</v>
       </c>
-      <c r="G43" t="s">
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="H43" cm="1">
+      <c r="H43" s="9" cm="1">
         <f t="array" ref="H43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score], StudentsPerformance[parental level of education]='Score Graphs'!$H$40))</f>
         <v>73.381355932203391</v>
       </c>
-      <c r="I43" cm="1">
+      <c r="I43" s="9" cm="1">
         <f t="array" ref="I43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score], StudentsPerformance[parental level of education]='Score Graphs'!$I$40))</f>
         <v>68.840707964601776</v>
       </c>
-      <c r="J43" cm="1">
+      <c r="J43" s="9" cm="1">
         <f t="array" ref="J43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score], StudentsPerformance[parental level of education]='Score Graphs'!$J$40))</f>
         <v>75.677966101694921</v>
       </c>
-      <c r="K43" cm="1">
+      <c r="K43" s="9" cm="1">
         <f t="array" ref="K43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score], StudentsPerformance[parental level of education]='Score Graphs'!$K$40))</f>
         <v>69.896396396396398</v>
       </c>
-      <c r="L43" cm="1">
+      <c r="L43" s="9" cm="1">
         <f t="array" ref="L43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score], StudentsPerformance[parental level of education]='Score Graphs'!$L$40))</f>
         <v>62.448979591836732</v>
       </c>
-      <c r="M43" cm="1">
+      <c r="M43" s="9" cm="1">
         <f t="array" ref="M43">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[writing score], StudentsPerformance[parental level of education]='Score Graphs'!$M$40))</f>
         <v>64.888268156424587</v>
       </c>
-    </row>
-    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B44" t="s">
+      <c r="N43" s="9"/>
+      <c r="O43" s="9"/>
+      <c r="Q43" s="9"/>
+      <c r="R43" s="9"/>
+      <c r="S43" s="9"/>
+      <c r="T43" s="9"/>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A44" s="9"/>
+      <c r="B44" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="C44" s="2" cm="1">
+      <c r="C44" s="10" cm="1">
         <f t="array" ref="C44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score],StudentsPerformance[gender]="male"))</f>
         <v>65.473029045643159</v>
       </c>
-      <c r="D44" s="2" cm="1">
+      <c r="D44" s="10" cm="1">
         <f t="array" ref="D44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score],StudentsPerformance[gender]="female"))</f>
         <v>72.608108108108112</v>
       </c>
-      <c r="G44" t="s">
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H44" cm="1">
+      <c r="H44" s="9" cm="1">
         <f t="array" ref="H44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score], StudentsPerformance[parental level of education]='Score Graphs'!$H$40))</f>
         <v>73</v>
       </c>
-      <c r="I44" cm="1">
+      <c r="I44" s="9" cm="1">
         <f t="array" ref="I44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score], StudentsPerformance[parental level of education]='Score Graphs'!$I$40))</f>
         <v>69.460176991150448</v>
       </c>
-      <c r="J44" cm="1">
+      <c r="J44" s="9" cm="1">
         <f t="array" ref="J44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score], StudentsPerformance[parental level of education]='Score Graphs'!$J$40))</f>
         <v>75.372881355932208</v>
       </c>
-      <c r="K44" cm="1">
+      <c r="K44" s="9" cm="1">
         <f t="array" ref="K44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score], StudentsPerformance[parental level of education]='Score Graphs'!$K$40))</f>
         <v>70.927927927927925</v>
       </c>
-      <c r="L44" cm="1">
+      <c r="L44" s="9" cm="1">
         <f t="array" ref="L44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score], StudentsPerformance[parental level of education]='Score Graphs'!$L$40))</f>
         <v>64.704081632653057</v>
       </c>
-      <c r="M44" cm="1">
+      <c r="M44" s="9" cm="1">
         <f t="array" ref="M44">AVERAGE(_xlfn._xlws.FILTER(StudentsPerformance[reading score], StudentsPerformance[parental level of education]='Score Graphs'!$M$40))</f>
         <v>66.938547486033514</v>
       </c>
+      <c r="N44" s="9"/>
+      <c r="O44" s="9"/>
+      <c r="P44" s="9"/>
+      <c r="Q44" s="9"/>
+      <c r="R44" s="9"/>
+      <c r="S44" s="9"/>
+      <c r="T44" s="9"/>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A45" s="9"/>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9"/>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+      <c r="I45" s="9"/>
+      <c r="J45" s="9"/>
+      <c r="K45" s="9"/>
+      <c r="L45" s="9"/>
+      <c r="M45" s="9"/>
+      <c r="N45" s="9"/>
+      <c r="O45" s="9"/>
+      <c r="P45" s="9"/>
+      <c r="Q45" s="9"/>
+      <c r="R45" s="9"/>
+      <c r="S45" s="9"/>
+      <c r="T45" s="9"/>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="A46" s="9"/>
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="9"/>
+      <c r="J46" s="9"/>
+      <c r="K46" s="9"/>
+      <c r="L46" s="9"/>
+      <c r="M46" s="9"/>
+      <c r="N46" s="9"/>
+      <c r="O46" s="9"/>
+      <c r="P46" s="9"/>
+      <c r="Q46" s="9"/>
+      <c r="R46" s="9"/>
+      <c r="S46" s="9"/>
+      <c r="T46" s="9"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>